<commit_message>
More control in index page
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghe/Documents/GitHub/drganghe.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6BA96E-4C0E-1C45-84A5-A57B9B930250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{890B6DE5-0D0D-6A41-8CA0-420B20C46551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="717">
   <si>
     <t>Section</t>
   </si>
@@ -394,9 +394,6 @@
     <t>https://github.com/drganghe/Rapid-and-Just-Coal-Transition-in-China</t>
   </si>
   <si>
-    <t>[SBU News](https://news.stonybrook.edu/homespotlight/study-shows-huge-benefits-of-transitioning-away-from-coal-in-china/) | [*Nature* News](https://www.nature.com/articles/d41586-020-02927-9)</t>
-  </si>
-  <si>
     <t>Coal Transition Network | Peking University</t>
   </si>
   <si>
@@ -1198,9 +1195,6 @@
     <t>https://drganghe.github.io/files/papers/2022-SPC-CarbonEmissionAndStructureAnalysisOfTransport.pdf</t>
   </si>
   <si>
-    <t>2022, peer-reviewed</t>
-  </si>
-  <si>
     <t>2022-05-01</t>
   </si>
   <si>
@@ -1876,27 +1870,15 @@
     <t>2026, peer-reviewed, power-system, china, grid-path</t>
   </si>
   <si>
-    <t>2022, selected, peer-reviewed, award, highly-cited, hot-paper, nature-series, supply-chain, solar, united-states, china, germany</t>
-  </si>
-  <si>
     <t>2022, selected, peer-reviewed, highly-cited, hot-paper, nature-series, china, carbon</t>
   </si>
   <si>
     <t>2021, selected, peer-reviewed, wind, AI</t>
   </si>
   <si>
-    <t>2017, selected, peer-reviewed, power-system</t>
-  </si>
-  <si>
     <t>2015, selected, peer-reviewed, china, city</t>
   </si>
   <si>
-    <t>2014, selected, peer-reviewed, china, wind</t>
-  </si>
-  <si>
-    <t>2013, selected, peer-reviewed, china, carbon</t>
-  </si>
-  <si>
     <t>2026, peer-reviewed, building, waste</t>
   </si>
   <si>
@@ -1918,9 +1900,6 @@
     <t>2022, peer-reviewed, behavior</t>
   </si>
   <si>
-    <t>2021, peer-reviewed, energy-efficiency</t>
-  </si>
-  <si>
     <t>2021, peer-reviewed, power-system, water</t>
   </si>
   <si>
@@ -1942,36 +1921,18 @@
     <t>2020, peer-reviewed, electricity, demand</t>
   </si>
   <si>
-    <t>2020, peer-reviewed, waste</t>
-  </si>
-  <si>
     <t>2020, peer-reviewed, water, electricity</t>
   </si>
   <si>
-    <t>2019, peer-reviewed, power-system, electricity, heat, natural-gas</t>
-  </si>
-  <si>
-    <t>2019, peer-reviewed, electricity, china</t>
-  </si>
-  <si>
     <t>2019, peer-reviewed, carbon</t>
   </si>
   <si>
-    <t>2018, peer-reviewed, industry, carbon</t>
-  </si>
-  <si>
     <t>2018, peer-reviewed, nuclear</t>
   </si>
   <si>
-    <t>2017, peer-reviewed, coal, china</t>
-  </si>
-  <si>
     <t>2017, peer-reviewed, power-system</t>
   </si>
   <si>
-    <t>2016, peer-reviewed, electricity, demand</t>
-  </si>
-  <si>
     <t>2013, peer-reviewed, building, industry</t>
   </si>
   <si>
@@ -1981,27 +1942,9 @@
     <t>2023, peer-reviewed, nature-series, energy-nexus, water, carbon</t>
   </si>
   <si>
-    <t>2025, selected, nature-series, power-system, china, supply-chain, nuclear</t>
-  </si>
-  <si>
-    <t>2016, selected, peer-reviewed, highly-cited, china, solar</t>
-  </si>
-  <si>
-    <t>2020, selected, peer-reviewed, china, coal, just-transition</t>
-  </si>
-  <si>
     <t>2018, peer-reviewed, water, energy-nexus</t>
   </si>
   <si>
-    <t>2023, peer-reviewed, nature-series, power-system, china, storage, switch-china</t>
-  </si>
-  <si>
-    <t>2016, selected, peer-reviewed, power-system, switch-china</t>
-  </si>
-  <si>
-    <t>2021, peer-reviewed, energy-nexus, power-system, water, switch-china</t>
-  </si>
-  <si>
     <t>2025, peer-reviewed, power-system, china, storage, grid-path</t>
   </si>
   <si>
@@ -2050,12 +1993,6 @@
     <t>Avrin, Anne-Perrine, **Gang He**, Daniel M. Kammen\*</t>
   </si>
   <si>
-    <t>2025, selected, peer-reviewed, solar, supply-chain, energy-nexus, united-states, health, climate, carbon</t>
-  </si>
-  <si>
-    <t>2017, selected, peer-reviewed, china, electricity</t>
-  </si>
-  <si>
     <t>2022, peer-reviewed, power-system</t>
   </si>
   <si>
@@ -2065,18 +2002,9 @@
     <t>2023, peer-reviewed, nature-series, supply-chain, carbon, solar, lca</t>
   </si>
   <si>
-    <t>2020, selected, peer-reviewed, highly-cited, nature-series, power-system, switch-china, solar, wind, storage</t>
-  </si>
-  <si>
     <t>2024, peer-reviewed, award, hydrogen, power-system, switch-china, lca</t>
   </si>
   <si>
-    <t>2020, peer-reviewed, waste, lca</t>
-  </si>
-  <si>
-    <t>2026, selected, power-system, AI</t>
-  </si>
-  <si>
     <t>2024, peer-reviewed, just-transition, energy-nexus, health</t>
   </si>
   <si>
@@ -2098,9 +2026,6 @@
     <t>https://ars.els-cdn.com/content/image/1-s2.0-S0921344916300957-mmc1.docx</t>
   </si>
   <si>
-    <t>2022, peer-reviewed, industry, carbon, transport</t>
-  </si>
-  <si>
     <t>2023, selected, peer-reviewed, highly-cited, hot-paper, nature-series, climate, solar, wind</t>
   </si>
   <si>
@@ -2116,19 +2041,194 @@
     <t>Zhang, Yang, Hongtao Bai, Huimin Hou, Yi Zhang, He Xu\*, Yijun Ji\*, **Gang He**, and Yingxuan Zhang</t>
   </si>
   <si>
-    <t>Cell Press 2024 China [Annual Paper](https://mp.weixin.qq.com/s/ZuXip64ASEsaJUDDfO_3bg) in the Sustainable Development Category</t>
-  </si>
-  <si>
     <t>2024, peer-reviewed, award, china, just-transition, coal</t>
+  </si>
+  <si>
+    <t>Cell Press 2024 China [Annual Papers](https://mp.weixin.qq.com/s/ZuXip64ASEsaJUDDfO_3bg) in the Sustainable Development Category</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-21-august-2025-chinas-co2-decline-two-mountains-chinas-cement-challenge/)</t>
+  </si>
+  <si>
+    <t>[SBU News](https://news.stonybrook.edu/homespotlight/study-shows-huge-benefits-of-transitioning-away-from-coal-in-china/) | [*Nature* News](https://www.nature.com/articles/d41586-020-02927-9) | [The Diplomat](https://thediplomat.com/2021/12/india-and-china-can-quit-coal-earlier-but-the-world-must-work-alongside-them/) | [Eco-Business](https://www.eco-business.com/news/health-and-climate-risks-overlap-in-coal-burning-southeast-asia/)</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-15-june-cbam-fight-new-energy-milestone-extreme-heat/)</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-17-february-2022-new-energy-transition-guidance-five-coal-plants-approved-energy-efficiency-targets-raised/)</t>
+  </si>
+  <si>
+    <t>[PKU News](https://news.pku.edu.cn/jxky/0d1098aa267a4ddfa1908784ff023570.htm) | [SBU News](https://news.stonybrook.edu/newsroom/taking-a-global-look-at-dry-and-alternative-water-cooling-of-power-plants/)</t>
+  </si>
+  <si>
+    <t>[THU News](https://www.tsinghua.edu.cn/info/1175/107135.htm)</t>
+  </si>
+  <si>
+    <t>[State of the Planet](https://news.climate.columbia.edu/2024/10/31/how-climate-change-impacts-affect-renewable-energy/) | [PKU News](https://news.pku.edu.cn/jxky/2d853f8a7dc544bca53aca9143e8085a.htm)</t>
+  </si>
+  <si>
+    <t>Peng, Liqun, **Gang He**, Nikit Abhyankar, Haozhe Yang, Umed Paliwal, and Jiang Lin\*</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Aligning offshore wind deployment with local priorities to accelerate power system decarbonization</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s43247-026-03533-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Communications Earth &amp; Environment </t>
+  </si>
+  <si>
+    <t>10.1038/s43247-026-03533-9</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s43247-026-03533-9.pdf</t>
+  </si>
+  <si>
+    <t>https://static-content.springer.com/esm/art%3A10.1038%2Fs43247-026-03533-9/MediaObjects/43247_2026_3533_MOESM2_ESM.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5281/zenodo.19375841</t>
+  </si>
+  <si>
+    <t>2026, nature-series, wind, power-system, grid-path</t>
+  </si>
+  <si>
+    <t>2026, first-author, corresponding-author, selected, nature-series, power-system, AI</t>
+  </si>
+  <si>
+    <t>2025, selected, corresponding-author, peer-reviewed, solar, supply-chain, energy-nexus, united-states, health, climate, carbon</t>
+  </si>
+  <si>
+    <t>2025, selected, corresponding-author, nature-series, power-system, china, supply-chain, nuclear</t>
+  </si>
+  <si>
+    <t>2022, selected, peer-reviewed, corresponding-author, award, highly-cited, hot-paper, nature-series, supply-chain, solar, united-states, china, germany</t>
+  </si>
+  <si>
+    <t>2020, selected, peer-reviewed, first-author, corresponding-author, highly-cited, nature-series, power-system, switch-china, solar, wind, storage</t>
+  </si>
+  <si>
+    <t>2020, selected, peer-reviewed, first-author, corresponding-author, china, coal, just-transition</t>
+  </si>
+  <si>
+    <t>2017, selected, peer-reviewed, first-author, corresponding-author, china, electricity</t>
+  </si>
+  <si>
+    <t>2017, selected, first-author, corresponding-author, peer-reviewed, power-system</t>
+  </si>
+  <si>
+    <t>2016, selected, peer-reviewed, first-author, corresponding-author, power-system, switch-china</t>
+  </si>
+  <si>
+    <t>2016, selected, peer-reviewed, first-author, corresponding-author, highly-cited, china, solar</t>
+  </si>
+  <si>
+    <t>2014, selected, peer-reviewed, first-author, corresponding-author, china, wind</t>
+  </si>
+  <si>
+    <t>2013, selected, peer-reviewed, first-author, corresponding-author, china, carbon</t>
+  </si>
+  <si>
+    <t>2023, peer-reviewed, corresponding-author, nature-series, power-system, china, storage, switch-china</t>
+  </si>
+  <si>
+    <t>2022, peer-reviewed, corresponding-author, industry, carbon, transport</t>
+  </si>
+  <si>
+    <t>2022, peer-reviewed, corresponding-author</t>
+  </si>
+  <si>
+    <t>2021, peer-reviewed, corresponding-author, energy-nexus, power-system, water, switch-china</t>
+  </si>
+  <si>
+    <t>2021, peer-reviewed, corresponding-author, energy-efficiency</t>
+  </si>
+  <si>
+    <t>2020, peer-reviewed, corresponding-author, waste, lca</t>
+  </si>
+  <si>
+    <t>2020, peer-reviewed, corresponding-author, waste</t>
+  </si>
+  <si>
+    <t>2019, peer-reviewed, corresponding-author, power-system, electricity, heat, natural-gas</t>
+  </si>
+  <si>
+    <t>2019, peer-reviewed, first-author, corresponding-author, electricity, china</t>
+  </si>
+  <si>
+    <t>2018, peer-reviewed, corresponding-author, industry, carbon</t>
+  </si>
+  <si>
+    <t>2017, peer-reviewed, corresponding-author, power-system</t>
+  </si>
+  <si>
+    <t>2017, peer-reviewed, corresponding-author, coal, china</t>
+  </si>
+  <si>
+    <t>2016, peer-reviewed, corresponding-author, electricity, demand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2274,13 +2374,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2291,8 +2398,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2599,7 +2709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X68"/>
+  <dimension ref="A1:X69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" style="1" customWidth="1"/>
@@ -2736,8 +2846,8 @@
       <c r="N2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="X2" s="11" t="s">
-        <v>684</v>
+      <c r="X2" s="25" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2783,8 +2893,8 @@
       <c r="V3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="X3" s="9" t="s">
-        <v>676</v>
+      <c r="X3" s="25" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2833,8 +2943,8 @@
       <c r="V4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="X4" s="5" t="s">
-        <v>653</v>
+      <c r="X4" s="25" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2886,8 +2996,11 @@
       <c r="T5" s="1">
         <v>1</v>
       </c>
-      <c r="X5" s="15" t="s">
-        <v>693</v>
+      <c r="V5" s="21" t="s">
+        <v>681</v>
+      </c>
+      <c r="X5" s="13" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2931,7 +3044,7 @@
         <v>80</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>687</v>
+        <v>663</v>
       </c>
       <c r="S6" s="1">
         <v>1</v>
@@ -2948,8 +3061,8 @@
       <c r="W6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="X6" s="5" t="s">
-        <v>618</v>
+      <c r="X6" s="26" t="s">
+        <v>695</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3002,7 +3115,7 @@
         <v>94</v>
       </c>
       <c r="X7" s="5" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3040,7 +3153,7 @@
         <v>103</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3095,8 +3208,8 @@
       <c r="W9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="X9" s="10" t="s">
-        <v>681</v>
+      <c r="X9" s="26" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3139,14 +3252,14 @@
       <c r="P10" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="V10" s="18" t="s">
+        <v>676</v>
+      </c>
+      <c r="W10" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="W10" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="X10" s="7" t="s">
-        <v>655</v>
+      <c r="X10" s="26" t="s">
+        <v>697</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3154,40 +3267,40 @@
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C11" s="1">
         <v>2017</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="K11" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="M11" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="W11" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="W11" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="X11" s="9" t="s">
-        <v>677</v>
+      <c r="X11" s="26" t="s">
+        <v>698</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3195,37 +3308,37 @@
         <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C12" s="1">
         <v>2017</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="L12" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="X12" s="5" t="s">
-        <v>621</v>
+      <c r="X12" s="26" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3233,49 +3346,49 @@
         <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C13" s="1">
         <v>2016</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>42</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="L13" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="O13" s="3" t="s">
-        <v>663</v>
+        <v>644</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>113</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="X13" s="7" t="s">
-        <v>658</v>
+        <v>152</v>
+      </c>
+      <c r="X13" s="26" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3283,43 +3396,43 @@
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C14" s="1">
         <v>2016</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="R14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="S14" s="1">
         <v>1</v>
       </c>
-      <c r="X14" s="6" t="s">
-        <v>654</v>
+      <c r="X14" s="26" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3327,43 +3440,43 @@
         <v>24</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C15" s="1">
         <v>2015</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="Q15" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="V15" t="s">
         <v>173</v>
       </c>
-      <c r="V15" t="s">
-        <v>174</v>
-      </c>
       <c r="X15" s="5" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3371,40 +3484,41 @@
         <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C16" s="1">
         <v>2014</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="L16" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="P16" s="3"/>
+      <c r="R16" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="R16" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="X16" s="5" t="s">
-        <v>623</v>
+      <c r="X16" s="26" t="s">
+        <v>702</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3412,2107 +3526,2163 @@
         <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C17" s="1">
         <v>2013</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="K17" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="L17" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="V17" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="V17" s="1" t="s">
+      <c r="W17" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="W17" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="X17" s="5" t="s">
-        <v>624</v>
+      <c r="X17" s="26" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>665</v>
+        <v>194</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>682</v>
       </c>
       <c r="C18" s="1">
         <v>2026</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>204</v>
+      <c r="D18" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>684</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>685</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>686</v>
+      </c>
+      <c r="K18" s="22" t="s">
+        <v>687</v>
+      </c>
+      <c r="L18" t="s">
+        <v>688</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>689</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="X18" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="R18" s="3" t="s">
         <v>690</v>
+      </c>
+      <c r="X18" s="24" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>205</v>
+        <v>194</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>646</v>
       </c>
       <c r="C19" s="1">
         <v>2026</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>89</v>
+        <v>199</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="X19" s="1" t="s">
-        <v>215</v>
+        <v>201</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="X19" s="12" t="s">
+        <v>666</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="C20" s="1">
         <v>2026</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>26</v>
+        <v>205</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>189</v>
+        <v>209</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="R20" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="X20" s="5" t="s">
-        <v>617</v>
+        <v>212</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="X20" s="1" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C21" s="1">
         <v>2026</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>225</v>
+        <v>26</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>229</v>
+        <v>188</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="X21" s="7" t="s">
-        <v>625</v>
+        <v>220</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="X21" s="5" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="C22" s="1">
         <v>2026</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>99</v>
+        <v>227</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="X22" s="5" t="s">
-        <v>626</v>
+        <v>230</v>
+      </c>
+      <c r="X22" s="6" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C23" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>209</v>
+        <v>99</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="O23" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="P23" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="R23" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="X23" s="7" t="s">
-        <v>661</v>
+        <v>237</v>
+      </c>
+      <c r="X23" s="5" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="C24" s="1">
         <v>2025</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>254</v>
+        <v>208</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="O24" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="X24" s="5" t="s">
-        <v>627</v>
+        <v>246</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="P24" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="X24" s="6" t="s">
+        <v>642</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="C25" s="1">
         <v>2025</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>130</v>
+        <v>253</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>265</v>
+        <v>254</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>255</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>268</v>
+        <v>258</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>259</v>
       </c>
       <c r="X25" s="5" t="s">
-        <v>628</v>
+        <v>621</v>
       </c>
     </row>
     <row r="26" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="C26" s="1">
         <v>2025</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>273</v>
+        <v>129</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="X26" s="7" t="s">
-        <v>660</v>
+        <v>266</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="V26" s="18" t="s">
+        <v>675</v>
+      </c>
+      <c r="X26" s="5" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="C27" s="1">
         <v>2025</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>209</v>
+        <v>272</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>243</v>
+        <v>273</v>
       </c>
       <c r="I27" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>284</v>
-      </c>
       <c r="K27" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="X27" s="12" t="s">
-        <v>689</v>
+        <v>276</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="X27" s="6" t="s">
+        <v>641</v>
       </c>
     </row>
     <row r="28" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="C28" s="1">
         <v>2025</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>291</v>
+        <v>208</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>292</v>
+        <v>242</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>31</v>
+        <v>274</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="X28" s="9" t="s">
-        <v>679</v>
+        <v>285</v>
+      </c>
+      <c r="X28" s="11" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="C29" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>40</v>
+        <v>290</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="R29" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="U29" s="18" t="s">
-        <v>698</v>
-      </c>
-      <c r="X29" s="18" t="s">
-        <v>699</v>
+        <v>294</v>
+      </c>
+      <c r="X29" s="8" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="30" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C30" s="1">
         <v>2024</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>310</v>
+        <v>40</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>31</v>
+        <v>299</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="P30" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="Q30" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="R30" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="X30" s="11" t="s">
-        <v>685</v>
+        <v>302</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="U30" s="17" t="s">
+        <v>674</v>
+      </c>
+      <c r="X30" s="16" t="s">
+        <v>673</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C31" s="1">
         <v>2024</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>148</v>
+        <v>309</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>321</v>
+        <v>31</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>244</v>
+        <v>30</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="U31" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="X31" s="11" t="s">
-        <v>682</v>
+        <v>313</v>
+      </c>
+      <c r="Q31" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="R31" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="X31" s="10" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="32" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C32" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>332</v>
+        <v>147</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>275</v>
+        <v>320</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>243</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>694</v>
-      </c>
-      <c r="R32" s="3" t="s">
-        <v>336</v>
+        <v>324</v>
+      </c>
+      <c r="P32" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="U32" s="1" t="s">
+        <v>326</v>
       </c>
       <c r="X32" s="10" t="s">
-        <v>680</v>
+        <v>660</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="C33" s="1">
         <v>2023</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>209</v>
+        <v>331</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="X33" s="5" t="s">
-        <v>629</v>
+        <v>669</v>
+      </c>
+      <c r="R33" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="V33" s="20" t="s">
+        <v>680</v>
+      </c>
+      <c r="X33" s="9" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="34" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="C34" s="1">
         <v>2023</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>108</v>
+        <v>208</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>350</v>
+        <v>340</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>255</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>664</v>
-      </c>
-      <c r="P34" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="X34" s="8" t="s">
-        <v>657</v>
+        <v>344</v>
+      </c>
+      <c r="X34" s="5" t="s">
+        <v>623</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="C35" s="1">
         <v>2023</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>359</v>
+        <v>108</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>41</v>
+        <v>349</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>362</v>
+        <v>351</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>352</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>363</v>
+        <v>645</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="X35" s="5" t="s">
-        <v>652</v>
+        <v>353</v>
+      </c>
+      <c r="X35" s="26" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="36" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="C36" s="1">
         <v>2023</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>370</v>
+        <v>31</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="X36" s="8" t="s">
-        <v>662</v>
+        <v>360</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="V36" s="20" t="s">
+        <v>679</v>
+      </c>
+      <c r="X36" s="5" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="C37" s="1">
         <v>2023</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>148</v>
+        <v>368</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>300</v>
+        <v>369</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="P37" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="X37" s="11" t="s">
-        <v>686</v>
+        <v>372</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>643</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="C38" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>387</v>
+        <v>147</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>388</v>
+        <v>377</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>299</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="X38" s="14" t="s">
-        <v>692</v>
+        <v>380</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="P38" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="V38" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="X38" s="10" t="s">
+        <v>662</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>695</v>
+        <v>194</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>382</v>
       </c>
       <c r="C39" s="1">
         <v>2022</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>130</v>
+        <v>386</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="S39" s="1">
-        <v>1</v>
-      </c>
-      <c r="X39" s="5" t="s">
-        <v>651</v>
+        <v>390</v>
+      </c>
+      <c r="X39" s="26" t="s">
+        <v>705</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>400</v>
+        <v>194</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>670</v>
       </c>
       <c r="C40" s="1">
         <v>2022</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>254</v>
+        <v>129</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>30</v>
+        <v>394</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="X40" s="9" t="s">
-        <v>678</v>
+        <v>397</v>
+      </c>
+      <c r="S40" s="1">
+        <v>1</v>
+      </c>
+      <c r="X40" s="5" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="C41" s="1">
         <v>2022</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>148</v>
+        <v>253</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>30</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="X41" s="5" t="s">
-        <v>630</v>
+        <v>405</v>
+      </c>
+      <c r="V41" s="19" t="s">
+        <v>678</v>
+      </c>
+      <c r="X41" s="8" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="42" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="C42" s="1">
         <v>2022</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>421</v>
+        <v>147</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>321</v>
+        <v>410</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>30</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="X42" s="1" t="s">
-        <v>425</v>
+        <v>413</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="X42" s="5" t="s">
+        <v>624</v>
       </c>
     </row>
     <row r="43" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="C43" s="1">
         <v>2022</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>431</v>
+        <v>320</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="X43" s="1" t="s">
-        <v>392</v>
+        <v>423</v>
       </c>
     </row>
     <row r="44" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>666</v>
+        <v>194</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>424</v>
       </c>
       <c r="C44" s="1">
         <v>2022</v>
       </c>
       <c r="D44" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>436</v>
-      </c>
       <c r="G44" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>89</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="X44" s="5" t="s">
-        <v>631</v>
+        <v>432</v>
+      </c>
+      <c r="X44" s="26" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="45" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>440</v>
+        <v>194</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>647</v>
       </c>
       <c r="C45" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>441</v>
+        <v>425</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>443</v>
+        <v>434</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>99</v>
+        <v>428</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>444</v>
+        <v>429</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="P45" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="X45" s="7" t="s">
-        <v>659</v>
+        <v>437</v>
+      </c>
+      <c r="X45" s="5" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="46" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>449</v>
+        <v>438</v>
       </c>
       <c r="C46" s="1">
         <v>2021</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>450</v>
+        <v>439</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>453</v>
+        <v>99</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>454</v>
+        <v>442</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="X46" s="5" t="s">
-        <v>632</v>
+        <v>444</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="X46" s="26" t="s">
+        <v>707</v>
       </c>
     </row>
     <row r="47" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="C47" s="1">
         <v>2021</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>459</v>
+        <v>449</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>199</v>
+        <v>451</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>461</v>
+        <v>452</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>462</v>
+        <v>453</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="L47" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="O47" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="X47" s="5" t="s">
-        <v>633</v>
+        <v>454</v>
+      </c>
+      <c r="X47" s="26" t="s">
+        <v>708</v>
       </c>
     </row>
     <row r="48" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>466</v>
+        <v>455</v>
       </c>
       <c r="C48" s="1">
         <v>2021</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>467</v>
+        <v>456</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>468</v>
+        <v>457</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>470</v>
+        <v>459</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>471</v>
+        <v>460</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>472</v>
+        <v>461</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>473</v>
+        <v>462</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="R48" s="1" t="s">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="X48" s="5" t="s">
-        <v>634</v>
+        <v>626</v>
       </c>
     </row>
     <row r="49" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>697</v>
+        <v>194</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>464</v>
       </c>
       <c r="C49" s="1">
         <v>2021</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>476</v>
+        <v>465</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>477</v>
+        <v>466</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>478</v>
+        <v>467</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>479</v>
+        <v>178</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>255</v>
+        <v>468</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>480</v>
+        <v>469</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>481</v>
+        <v>470</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="R49" s="1" t="s">
+        <v>473</v>
       </c>
       <c r="X49" s="5" t="s">
-        <v>635</v>
+        <v>627</v>
       </c>
     </row>
     <row r="50" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>482</v>
+        <v>194</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>672</v>
       </c>
       <c r="C50" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>487</v>
+        <v>254</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="L50" s="1" t="s">
-        <v>490</v>
+        <v>479</v>
       </c>
       <c r="X50" s="5" t="s">
-        <v>636</v>
+        <v>628</v>
       </c>
     </row>
     <row r="51" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B51" s="17" t="s">
-        <v>696</v>
+        <v>194</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>480</v>
       </c>
       <c r="C51" s="1">
         <v>2020</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>491</v>
+        <v>481</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>492</v>
+        <v>482</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>493</v>
+        <v>483</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>99</v>
+        <v>484</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
       <c r="X51" s="5" t="s">
-        <v>637</v>
+        <v>629</v>
       </c>
     </row>
     <row r="52" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>667</v>
+        <v>194</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>671</v>
       </c>
       <c r="C52" s="1">
         <v>2020</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
       <c r="X52" s="5" t="s">
-        <v>638</v>
+        <v>630</v>
       </c>
     </row>
     <row r="53" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>668</v>
+        <v>194</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>648</v>
       </c>
       <c r="C53" s="1">
         <v>2020</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>508</v>
+        <v>99</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>511</v>
+        <v>501</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>502</v>
       </c>
       <c r="X53" s="5" t="s">
-        <v>639</v>
+        <v>631</v>
       </c>
     </row>
     <row r="54" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B54" s="9" t="s">
-        <v>669</v>
+        <v>194</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>649</v>
       </c>
       <c r="C54" s="1">
         <v>2020</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>513</v>
+        <v>504</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>514</v>
+        <v>505</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>518</v>
-      </c>
-      <c r="X54" s="11" t="s">
-        <v>683</v>
+        <v>509</v>
+      </c>
+      <c r="X54" s="5" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="55" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>670</v>
+        <v>194</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>650</v>
       </c>
       <c r="C55" s="1">
         <v>2020</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>99</v>
+        <v>513</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="X55" s="5" t="s">
-        <v>640</v>
+        <v>516</v>
+      </c>
+      <c r="X55" s="26" t="s">
+        <v>709</v>
       </c>
     </row>
     <row r="56" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>525</v>
+        <v>194</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>651</v>
       </c>
       <c r="C56" s="1">
         <v>2020</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>526</v>
+        <v>517</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>527</v>
+        <v>518</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>528</v>
+        <v>519</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>529</v>
+        <v>520</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>530</v>
+        <v>521</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>531</v>
-      </c>
-      <c r="L56" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="X56" s="5" t="s">
-        <v>641</v>
+        <v>522</v>
+      </c>
+      <c r="X56" s="26" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="57" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="C57" s="1">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>453</v>
+        <v>99</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>539</v>
+        <v>529</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>530</v>
       </c>
       <c r="X57" s="5" t="s">
-        <v>642</v>
+        <v>633</v>
       </c>
     </row>
     <row r="58" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>25</v>
+        <v>194</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>531</v>
       </c>
       <c r="C58" s="1">
         <v>2019</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>543</v>
+        <v>451</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>31</v>
+        <v>535</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>536</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="X58" s="5" t="s">
-        <v>643</v>
+        <v>537</v>
+      </c>
+      <c r="X58" s="26" t="s">
+        <v>711</v>
       </c>
     </row>
     <row r="59" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B59" s="9" t="s">
-        <v>671</v>
+        <v>194</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="C59" s="1">
         <v>2019</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>550</v>
-      </c>
-      <c r="J59" s="1" t="s">
-        <v>551</v>
+        <v>41</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>553</v>
-      </c>
-      <c r="X59" s="5" t="s">
-        <v>644</v>
+        <v>543</v>
+      </c>
+      <c r="X59" s="26" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="60" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>672</v>
+        <v>194</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>652</v>
       </c>
       <c r="C60" s="1">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>555</v>
+        <v>545</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>556</v>
+        <v>546</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>99</v>
+        <v>547</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>557</v>
+        <v>548</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>559</v>
+        <v>550</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="X60" s="7" t="s">
-        <v>656</v>
+        <v>551</v>
+      </c>
+      <c r="X60" s="5" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="61" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>561</v>
+        <v>194</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>653</v>
       </c>
       <c r="C61" s="1">
         <v>2018</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>562</v>
+        <v>552</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>564</v>
+        <v>554</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>486</v>
+        <v>99</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>566</v>
+        <v>556</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>567</v>
+        <v>557</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>568</v>
-      </c>
-      <c r="X61" s="5" t="s">
-        <v>645</v>
+        <v>558</v>
+      </c>
+      <c r="X61" s="6" t="s">
+        <v>640</v>
       </c>
     </row>
     <row r="62" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B62" s="9" t="s">
-        <v>673</v>
+        <v>194</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>559</v>
       </c>
       <c r="C62" s="1">
         <v>2018</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>570</v>
+        <v>561</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>571</v>
+        <v>562</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>572</v>
+        <v>563</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>573</v>
+        <v>564</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="X62" s="5" t="s">
-        <v>646</v>
+        <v>565</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="X62" s="26" t="s">
+        <v>713</v>
       </c>
     </row>
     <row r="63" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>575</v>
+        <v>194</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>654</v>
       </c>
       <c r="C63" s="1">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>130</v>
+        <v>484</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="X63" s="5" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
     </row>
     <row r="64" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B64" s="9" t="s">
-        <v>674</v>
+        <v>194</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>573</v>
       </c>
       <c r="C64" s="1">
         <v>2017</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>453</v>
+        <v>129</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="K64" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="X64" s="5" t="s">
-        <v>648</v>
+        <v>579</v>
+      </c>
+      <c r="X64" s="26" t="s">
+        <v>715</v>
       </c>
     </row>
     <row r="65" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>588</v>
+        <v>194</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>655</v>
       </c>
       <c r="C65" s="1">
         <v>2017</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>589</v>
+        <v>580</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>590</v>
+        <v>581</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>591</v>
+        <v>582</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>130</v>
+        <v>451</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>140</v>
+        <v>583</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
       <c r="K65" s="1" t="s">
-        <v>593</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>691</v>
-      </c>
-      <c r="X65" s="5" t="s">
-        <v>648</v>
+        <v>585</v>
+      </c>
+      <c r="X65" s="26" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="66" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="C66" s="1">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>596</v>
+        <v>588</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>273</v>
+        <v>129</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>89</v>
+        <v>139</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>599</v>
+        <v>590</v>
       </c>
       <c r="K66" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="X66" s="5" t="s">
-        <v>649</v>
+        <v>591</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="X66" s="26" t="s">
+        <v>714</v>
       </c>
     </row>
     <row r="67" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>675</v>
+        <v>194</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>592</v>
       </c>
       <c r="C67" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>601</v>
+        <v>593</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>602</v>
+        <v>594</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>603</v>
+        <v>595</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>604</v>
+        <v>272</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>605</v>
+        <v>596</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="K67" s="1" t="s">
-        <v>607</v>
-      </c>
-      <c r="L67" s="1" t="s">
-        <v>608</v>
-      </c>
-      <c r="O67" s="1" t="s">
-        <v>609</v>
-      </c>
-      <c r="X67" s="1" t="s">
-        <v>610</v>
+        <v>598</v>
+      </c>
+      <c r="X67" s="26" t="s">
+        <v>716</v>
       </c>
     </row>
     <row r="68" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B68" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>656</v>
+      </c>
+      <c r="C68" s="1">
+        <v>2015</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="L68" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="O68" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="X68" s="1" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="69" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="C69" s="1">
+        <v>2013</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="E69" s="1" t="s">
         <v>611</v>
       </c>
-      <c r="C68" s="1">
-        <v>2013</v>
-      </c>
-      <c r="D68" s="2" t="s">
+      <c r="F69" s="1" t="s">
         <v>612</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="G69" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="J69" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="F68" s="1" t="s">
+      <c r="K69" s="1" t="s">
         <v>614</v>
       </c>
-      <c r="G68" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>615</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>616</v>
-      </c>
-      <c r="X68" s="5" t="s">
-        <v>650</v>
+      <c r="X69" s="5" t="s">
+        <v>637</v>
       </c>
     </row>
   </sheetData>
@@ -5521,20 +5691,24 @@
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="F10" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="P23" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="R23" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="P30" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="Q30" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="R30" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="R32" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="P34" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="P45" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="P24" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="R24" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="P31" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="Q31" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="R31" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="R33" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="P35" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="P46" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
     <hyperlink ref="O13" r:id="rId13" xr:uid="{E1B68A12-C2D1-2D4C-9BA7-D957598FA97F}"/>
-    <hyperlink ref="P37" r:id="rId14" xr:uid="{1F4DB385-82C7-B34A-952A-9E6D95022546}"/>
-    <hyperlink ref="P31" r:id="rId15" xr:uid="{F06DA3D7-59A8-D84B-93E1-440C92628887}"/>
+    <hyperlink ref="P38" r:id="rId14" xr:uid="{1F4DB385-82C7-B34A-952A-9E6D95022546}"/>
+    <hyperlink ref="P32" r:id="rId15" xr:uid="{F06DA3D7-59A8-D84B-93E1-440C92628887}"/>
     <hyperlink ref="R6" r:id="rId16" xr:uid="{3BA53A63-8360-5C4A-8B83-6B57EC2CA670}"/>
-    <hyperlink ref="O23" r:id="rId17" xr:uid="{DBD76148-39E2-0A4A-BEB0-0119C38CF222}"/>
-    <hyperlink ref="P18" r:id="rId18" xr:uid="{86409AA4-BEFD-D542-B873-480C74955AF8}"/>
+    <hyperlink ref="O24" r:id="rId17" xr:uid="{DBD76148-39E2-0A4A-BEB0-0119C38CF222}"/>
+    <hyperlink ref="P19" r:id="rId18" xr:uid="{86409AA4-BEFD-D542-B873-480C74955AF8}"/>
+    <hyperlink ref="F18" r:id="rId19" xr:uid="{D215DD66-92F0-B743-B8A1-3D4196786705}"/>
+    <hyperlink ref="O18" r:id="rId20" xr:uid="{1D7B2550-014B-C64E-AEB9-00BD366191E0}"/>
+    <hyperlink ref="P18" r:id="rId21" xr:uid="{5DE482F3-CFB9-9F4D-9BDA-A163AE0ADB50}"/>
+    <hyperlink ref="R18" r:id="rId22" xr:uid="{BFAA4559-24D5-B443-8FC5-A54634E39487}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
rerender to enable llms
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghe/Documents/GitHub/drganghe.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6BA96E-4C0E-1C45-84A5-A57B9B930250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B3E26D-2251-0340-BFD1-C70123B0A003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="705">
   <si>
     <t>Section</t>
   </si>
@@ -394,9 +394,6 @@
     <t>https://github.com/drganghe/Rapid-and-Just-Coal-Transition-in-China</t>
   </si>
   <si>
-    <t>[SBU News](https://news.stonybrook.edu/homespotlight/study-shows-huge-benefits-of-transitioning-away-from-coal-in-china/) | [*Nature* News](https://www.nature.com/articles/d41586-020-02927-9)</t>
-  </si>
-  <si>
     <t>Coal Transition Network | Peking University</t>
   </si>
   <si>
@@ -2116,19 +2113,58 @@
     <t>Zhang, Yang, Hongtao Bai, Huimin Hou, Yi Zhang, He Xu\*, Yijun Ji\*, **Gang He**, and Yingxuan Zhang</t>
   </si>
   <si>
-    <t>Cell Press 2024 China [Annual Paper](https://mp.weixin.qq.com/s/ZuXip64ASEsaJUDDfO_3bg) in the Sustainable Development Category</t>
-  </si>
-  <si>
     <t>2024, peer-reviewed, award, china, just-transition, coal</t>
+  </si>
+  <si>
+    <t>Cell Press 2024 China [Annual Papers](https://mp.weixin.qq.com/s/ZuXip64ASEsaJUDDfO_3bg) in the Sustainable Development Category</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-21-august-2025-chinas-co2-decline-two-mountains-chinas-cement-challenge/)</t>
+  </si>
+  <si>
+    <t>[SBU News](https://news.stonybrook.edu/homespotlight/study-shows-huge-benefits-of-transitioning-away-from-coal-in-china/) | [*Nature* News](https://www.nature.com/articles/d41586-020-02927-9) | [The Diplomat](https://thediplomat.com/2021/12/india-and-china-can-quit-coal-earlier-but-the-world-must-work-alongside-them/) | [Eco-Business](https://www.eco-business.com/news/health-and-climate-risks-overlap-in-coal-burning-southeast-asia/)</t>
+  </si>
+  <si>
+    <t>[Tsinghua University](https://www.tsinghua.edu.cn/info/1175/107135.htm)</t>
+  </si>
+  <si>
+    <t>[Peking University](https://news.pku.edu.cn/jxky/0d1098aa267a4ddfa1908784ff023570.htm) | [Stony Brook University](https://news.stonybrook.edu/newsroom/taking-a-global-look-at-dry-and-alternative-water-cooling-of-power-plants/)</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-15-june-cbam-fight-new-energy-milestone-extreme-heat/)</t>
+  </si>
+  <si>
+    <t>[Carbon Brief](https://www.carbonbrief.org/china-briefing-17-february-2022-new-energy-transition-guidance-five-coal-plants-approved-energy-efficiency-targets-raised/)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2274,13 +2310,16 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2737,7 +2776,7 @@
         <v>35</v>
       </c>
       <c r="X2" s="11" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2784,7 +2823,7 @@
         <v>47</v>
       </c>
       <c r="X3" s="9" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2834,7 +2873,7 @@
         <v>60</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2887,7 +2926,7 @@
         <v>1</v>
       </c>
       <c r="X5" s="15" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -2931,7 +2970,7 @@
         <v>80</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="S6" s="1">
         <v>1</v>
@@ -2949,7 +2988,7 @@
         <v>83</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3002,7 +3041,7 @@
         <v>94</v>
       </c>
       <c r="X7" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3040,7 +3079,7 @@
         <v>103</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3096,7 +3135,7 @@
         <v>115</v>
       </c>
       <c r="X9" s="10" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3139,14 +3178,14 @@
       <c r="P10" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="V10" s="20" t="s">
+        <v>700</v>
+      </c>
+      <c r="W10" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="W10" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="X10" s="7" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3154,40 +3193,40 @@
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C11" s="1">
         <v>2017</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="K11" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="M11" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="W11" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="W11" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="X11" s="9" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3195,37 +3234,37 @@
         <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C12" s="1">
         <v>2017</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="L12" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="X12" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3233,49 +3272,49 @@
         <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C13" s="1">
         <v>2016</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>42</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="L13" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="O13" s="3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>113</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="X13" s="7" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3283,43 +3322,43 @@
         <v>24</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C14" s="1">
         <v>2016</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="R14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="S14" s="1">
         <v>1</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3327,43 +3366,43 @@
         <v>24</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C15" s="1">
         <v>2015</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="Q15" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="V15" t="s">
         <v>173</v>
       </c>
-      <c r="V15" t="s">
-        <v>174</v>
-      </c>
       <c r="X15" s="5" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3371,40 +3410,40 @@
         <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C16" s="1">
         <v>2014</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="L16" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="R16" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="X16" s="5" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="17" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -3412,139 +3451,139 @@
         <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C17" s="1">
         <v>2013</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="K17" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="L17" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="V17" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="V17" s="1" t="s">
+      <c r="W17" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="W17" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="X17" s="5" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="18" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C18" s="1">
         <v>2026</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="O18" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>113</v>
       </c>
       <c r="X18" s="13" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C19" s="1">
         <v>2026</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>89</v>
       </c>
       <c r="J19" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="L19" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="Q19" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="Q19" s="1" t="s">
+      <c r="X19" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="X19" s="1" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C20" s="1">
         <v>2026</v>
@@ -3553,432 +3592,435 @@
         <v>26</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="J20" s="1" t="s">
+      <c r="K20" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="L20" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="R20" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="R20" s="1" t="s">
-        <v>223</v>
-      </c>
       <c r="X20" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C21" s="1">
         <v>2026</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="K21" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>231</v>
-      </c>
       <c r="X21" s="7" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C22" s="1">
         <v>2026</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>235</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H22" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="J22" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>238</v>
-      </c>
       <c r="X22" s="5" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="23" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C23" s="1">
         <v>2025</v>
       </c>
       <c r="D23" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="L23" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="L23" s="1" t="s">
+      <c r="O23" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="P23" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="O23" s="3" t="s">
-        <v>688</v>
-      </c>
-      <c r="P23" s="3" t="s">
+      <c r="R23" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="R23" s="3" t="s">
-        <v>249</v>
-      </c>
       <c r="X23" s="7" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C24" s="1">
         <v>2025</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="H24" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="L24" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="O24" s="1" t="s">
-        <v>260</v>
-      </c>
       <c r="X24" s="5" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="25" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C25" s="1">
         <v>2025</v>
       </c>
       <c r="D25" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="G25" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="L25" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>268</v>
+      <c r="V25" s="20" t="s">
+        <v>699</v>
       </c>
       <c r="X25" s="5" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="26" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C26" s="1">
         <v>2025</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="M26" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="M26" s="1" t="s">
+      <c r="R26" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="R26" s="1" t="s">
-        <v>279</v>
-      </c>
       <c r="X26" s="7" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="27" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C27" s="1">
         <v>2025</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="J27" s="1" t="s">
+      <c r="K27" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="K27" s="1" t="s">
+      <c r="L27" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L27" s="1" t="s">
-        <v>286</v>
-      </c>
       <c r="X27" s="12" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="28" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C28" s="1">
         <v>2025</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="H28" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>292</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>31</v>
       </c>
       <c r="J28" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="K28" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="K28" s="1" t="s">
+      <c r="L28" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="L28" s="1" t="s">
-        <v>295</v>
-      </c>
       <c r="X28" s="9" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="29" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C29" s="1">
         <v>2024</v>
       </c>
       <c r="D29" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>298</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>299</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>40</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>42</v>
       </c>
       <c r="J29" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="K29" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="K29" s="1" t="s">
+      <c r="L29" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="L29" s="1" t="s">
+      <c r="O29" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="O29" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="R29" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="U29" s="18" t="s">
+      <c r="U29" s="19" t="s">
         <v>698</v>
       </c>
       <c r="X29" s="18" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
     </row>
     <row r="30" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C30" s="1">
         <v>2024</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>310</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>31</v>
@@ -3987,236 +4029,239 @@
         <v>30</v>
       </c>
       <c r="J30" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="K30" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="L30" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="P30" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="P30" s="3" t="s">
+      <c r="Q30" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="Q30" s="3" t="s">
+      <c r="R30" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="R30" s="3" t="s">
-        <v>316</v>
-      </c>
       <c r="X30" s="11" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="31" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C31" s="1">
         <v>2024</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="J31" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="J31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="L31" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="L31" s="1" t="s">
+      <c r="O31" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>325</v>
       </c>
       <c r="P31" s="3" t="s">
         <v>113</v>
       </c>
       <c r="R31" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="U31" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="U31" s="1" t="s">
-        <v>327</v>
-      </c>
       <c r="X31" s="11" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="32" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C32" s="1">
         <v>2023</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="H32" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="J32" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="H32" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="J32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="L32" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="O32" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="R32" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="O32" s="1" t="s">
-        <v>694</v>
-      </c>
-      <c r="R32" s="3" t="s">
-        <v>336</v>
+      <c r="V32" s="21" t="s">
+        <v>701</v>
       </c>
       <c r="X32" s="10" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C33" s="1">
         <v>2023</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H33" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H33" s="1" t="s">
+      <c r="I33" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="J33" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="J33" s="1" t="s">
+      <c r="K33" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="K33" s="1" t="s">
+      <c r="L33" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="L33" s="1" t="s">
+      <c r="O33" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="O33" s="1" t="s">
-        <v>345</v>
-      </c>
       <c r="X33" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="34" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C34" s="1">
         <v>2023</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>349</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>108</v>
       </c>
       <c r="H34" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="L34" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="L34" s="1" t="s">
-        <v>353</v>
-      </c>
       <c r="O34" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="P34" s="3" t="s">
         <v>113</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="X34" s="8" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C35" s="1">
         <v>2023</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>359</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>31</v>
@@ -4225,890 +4270,899 @@
         <v>41</v>
       </c>
       <c r="J35" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="K35" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="K35" s="1" t="s">
+      <c r="N35" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="N35" s="1" t="s">
+      <c r="O35" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="O35" s="1" t="s">
+      <c r="R35" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="R35" s="1" t="s">
-        <v>364</v>
+      <c r="V35" s="21" t="s">
+        <v>702</v>
       </c>
       <c r="X35" s="5" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="36" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C36" s="1">
         <v>2023</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="J36" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="K36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="L36" s="1" t="s">
-        <v>373</v>
-      </c>
       <c r="X36" s="8" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="37" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C37" s="1">
         <v>2023</v>
       </c>
       <c r="D37" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H37" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="J37" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="I37" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="J37" s="1" t="s">
+      <c r="K37" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="L37" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L37" s="1" t="s">
+      <c r="O37" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="O37" s="1" t="s">
-        <v>382</v>
-      </c>
       <c r="P37" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
+      </c>
+      <c r="V37" s="21" t="s">
+        <v>703</v>
       </c>
       <c r="X37" s="11" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="38" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C38" s="1">
         <v>2022</v>
       </c>
       <c r="D38" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="H38" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="J38" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="J38" s="1" t="s">
+      <c r="K38" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="L38" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="L38" s="1" t="s">
-        <v>391</v>
-      </c>
       <c r="X38" s="14" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="39" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C39" s="1">
         <v>2022</v>
       </c>
       <c r="D39" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="G39" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H39" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H39" s="1" t="s">
+      <c r="J39" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="J39" s="1" t="s">
+      <c r="K39" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="K39" s="1" t="s">
+      <c r="L39" s="1" t="s">
         <v>398</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>399</v>
       </c>
       <c r="S39" s="1">
         <v>1</v>
       </c>
       <c r="X39" s="5" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C40" s="1">
         <v>2022</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="H40" s="1" t="s">
         <v>403</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>404</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>30</v>
       </c>
       <c r="J40" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="K40" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="K40" s="1" t="s">
+      <c r="L40" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="L40" s="1" t="s">
-        <v>407</v>
+      <c r="V40" s="21" t="s">
+        <v>704</v>
       </c>
       <c r="X40" s="9" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="41" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C41" s="1">
         <v>2022</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G41" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="H41" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>412</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>30</v>
       </c>
       <c r="J41" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="K41" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="L41" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="L41" s="1" t="s">
+      <c r="O41" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="O41" s="1" t="s">
-        <v>416</v>
-      </c>
       <c r="X41" s="5" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="42" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C42" s="1">
         <v>2022</v>
       </c>
       <c r="D42" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E42" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>421</v>
-      </c>
       <c r="H42" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>30</v>
       </c>
       <c r="J42" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="K42" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="K42" s="1" t="s">
+      <c r="L42" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="L42" s="1" t="s">
+      <c r="X42" s="1" t="s">
         <v>424</v>
-      </c>
-      <c r="X42" s="1" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="43" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C43" s="1">
         <v>2022</v>
       </c>
       <c r="D43" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>430</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>431</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>89</v>
       </c>
       <c r="J43" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="K43" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="K43" s="1" t="s">
+      <c r="L43" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="L43" s="1" t="s">
-        <v>434</v>
-      </c>
       <c r="X43" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="44" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C44" s="1">
         <v>2022</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E44" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="F44" s="1" t="s">
-        <v>436</v>
-      </c>
       <c r="G44" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>430</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>431</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>89</v>
       </c>
       <c r="J44" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="K44" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="K44" s="1" t="s">
+      <c r="L44" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="L44" s="1" t="s">
-        <v>439</v>
-      </c>
       <c r="X44" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="45" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C45" s="1">
         <v>2021</v>
       </c>
       <c r="D45" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="F45" s="1" t="s">
         <v>442</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>443</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H45" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="J45" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="J45" s="1" t="s">
+      <c r="K45" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="K45" s="1" t="s">
+      <c r="L45" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="L45" s="1" t="s">
+      <c r="O45" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>448</v>
       </c>
       <c r="P45" s="3" t="s">
         <v>113</v>
       </c>
       <c r="X45" s="7" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="46" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C46" s="1">
         <v>2021</v>
       </c>
       <c r="D46" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="G46" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="H46" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="J46" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="K46" s="1" t="s">
-        <v>456</v>
-      </c>
       <c r="X46" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="47" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C47" s="1">
         <v>2021</v>
       </c>
       <c r="D47" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="G47" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H47" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="G47" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H47" s="1" t="s">
+      <c r="J47" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="K47" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="K47" s="1" t="s">
+      <c r="L47" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="L47" s="1" t="s">
+      <c r="O47" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="O47" s="1" t="s">
-        <v>465</v>
-      </c>
       <c r="X47" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="48" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C48" s="1">
         <v>2021</v>
       </c>
       <c r="D48" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="F48" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="G48" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H48" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="G48" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H48" s="1" t="s">
+      <c r="J48" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="J48" s="1" t="s">
+      <c r="K48" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="K48" s="1" t="s">
+      <c r="L48" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="L48" s="1" t="s">
+      <c r="O48" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="O48" s="1" t="s">
+      <c r="R48" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="R48" s="1" t="s">
-        <v>475</v>
-      </c>
       <c r="X48" s="5" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="49" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C49" s="1">
         <v>2021</v>
       </c>
       <c r="D49" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="F49" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="G49" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="G49" s="1" t="s">
+      <c r="H49" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="J49" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="H49" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="J49" s="1" t="s">
+      <c r="K49" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="K49" s="1" t="s">
-        <v>481</v>
-      </c>
       <c r="X49" s="5" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="50" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C50" s="1">
         <v>2020</v>
       </c>
       <c r="D50" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="G50" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="G50" s="1" t="s">
+      <c r="H50" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="J50" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="J50" s="1" t="s">
+      <c r="K50" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="K50" s="1" t="s">
+      <c r="L50" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="L50" s="1" t="s">
-        <v>490</v>
-      </c>
       <c r="X50" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="51" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C51" s="1">
         <v>2020</v>
       </c>
       <c r="D51" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="F51" s="1" t="s">
         <v>492</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>493</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H51" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="J51" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="J51" s="1" t="s">
+      <c r="K51" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="K51" s="1" t="s">
+      <c r="L51" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="L51" s="1" t="s">
-        <v>497</v>
-      </c>
       <c r="X51" s="5" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="52" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C52" s="1">
         <v>2020</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="F52" s="1" t="s">
         <v>499</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>500</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H52" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="J52" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="J52" s="1" t="s">
+      <c r="K52" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="K52" s="1" t="s">
+      <c r="L52" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="L52" s="1" t="s">
-        <v>504</v>
-      </c>
       <c r="X52" s="5" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="53" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C53" s="1">
         <v>2020</v>
       </c>
       <c r="D53" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="F53" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="H53" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="H53" s="1" t="s">
+      <c r="J53" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="J53" s="1" t="s">
+      <c r="K53" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="K53" s="1" t="s">
-        <v>511</v>
-      </c>
       <c r="X53" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="54" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C54" s="1">
         <v>2020</v>
       </c>
       <c r="D54" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="F54" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="G54" s="1" t="s">
+      <c r="H54" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="H54" s="1" t="s">
+      <c r="J54" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="J54" s="1" t="s">
+      <c r="K54" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="K54" s="1" t="s">
-        <v>518</v>
-      </c>
       <c r="X54" s="11" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="55" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="C55" s="1">
         <v>2020</v>
       </c>
       <c r="D55" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="F55" s="1" t="s">
         <v>520</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>521</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H55" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="J55" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="J55" s="1" t="s">
+      <c r="K55" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="K55" s="1" t="s">
-        <v>524</v>
-      </c>
       <c r="X55" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="56" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C56" s="1">
         <v>2020</v>
       </c>
       <c r="D56" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="E56" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="F56" s="1" t="s">
         <v>527</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>528</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H56" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="J56" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="J56" s="1" t="s">
+      <c r="K56" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="K56" s="1" t="s">
+      <c r="L56" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="L56" s="1" t="s">
-        <v>532</v>
-      </c>
       <c r="X56" s="5" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="57" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C57" s="1">
         <v>2019</v>
       </c>
       <c r="D57" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="F57" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="H57" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="H57" s="1" t="s">
+      <c r="J57" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="J57" s="1" t="s">
+      <c r="K57" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="K57" s="1" t="s">
-        <v>539</v>
-      </c>
       <c r="X57" s="5" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="58" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>25</v>
@@ -5117,16 +5171,16 @@
         <v>2019</v>
       </c>
       <c r="D58" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="F58" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="1" t="s">
         <v>542</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>543</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>41</v>
@@ -5135,384 +5189,384 @@
         <v>31</v>
       </c>
       <c r="K58" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="L58" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="L58" s="1" t="s">
-        <v>545</v>
-      </c>
       <c r="X58" s="5" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="59" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C59" s="1">
         <v>2019</v>
       </c>
       <c r="D59" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="G59" s="1" t="s">
+      <c r="H59" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="H59" s="1" t="s">
+      <c r="J59" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="J59" s="1" t="s">
+      <c r="K59" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="K59" s="1" t="s">
+      <c r="L59" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="L59" s="1" t="s">
-        <v>553</v>
-      </c>
       <c r="X59" s="5" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="60" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="C60" s="1">
         <v>2018</v>
       </c>
       <c r="D60" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="F60" s="1" t="s">
         <v>555</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>556</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>99</v>
       </c>
       <c r="H60" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="J60" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="J60" s="1" t="s">
+      <c r="K60" s="1" t="s">
         <v>558</v>
       </c>
-      <c r="K60" s="1" t="s">
+      <c r="L60" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="L60" s="1" t="s">
-        <v>560</v>
-      </c>
       <c r="X60" s="7" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="61" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C61" s="1">
         <v>2018</v>
       </c>
       <c r="D61" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="F61" s="1" t="s">
         <v>563</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="H61" s="1" t="s">
         <v>564</v>
       </c>
-      <c r="G61" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="H61" s="1" t="s">
+      <c r="J61" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="J61" s="1" t="s">
+      <c r="K61" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="K61" s="1" t="s">
+      <c r="L61" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="L61" s="1" t="s">
-        <v>568</v>
-      </c>
       <c r="X61" s="5" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="62" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="C62" s="1">
         <v>2018</v>
       </c>
       <c r="D62" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>569</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="F62" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="H62" s="1" t="s">
         <v>571</v>
       </c>
-      <c r="G62" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="H62" s="1" t="s">
+      <c r="J62" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="J62" s="1" t="s">
+      <c r="K62" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="K62" s="1" t="s">
-        <v>574</v>
-      </c>
       <c r="X62" s="5" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="63" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C63" s="1">
         <v>2017</v>
       </c>
       <c r="D63" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="F63" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="G63" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H63" s="1" t="s">
+      <c r="J63" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="J63" s="1" t="s">
+      <c r="K63" s="1" t="s">
         <v>580</v>
       </c>
-      <c r="K63" s="1" t="s">
-        <v>581</v>
-      </c>
       <c r="X63" s="5" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="64" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="C64" s="1">
         <v>2017</v>
       </c>
       <c r="D64" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="F64" s="1" t="s">
         <v>583</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="G64" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="H64" s="1" t="s">
+      <c r="J64" s="1" t="s">
         <v>585</v>
       </c>
-      <c r="J64" s="1" t="s">
+      <c r="K64" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="K64" s="1" t="s">
-        <v>587</v>
-      </c>
       <c r="X64" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="65" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C65" s="1">
         <v>2017</v>
       </c>
       <c r="D65" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>589</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="F65" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="G65" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J65" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="G65" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="J65" s="1" t="s">
+      <c r="K65" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="K65" s="1" t="s">
-        <v>593</v>
-      </c>
       <c r="O65" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="X65" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="66" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C66" s="1">
         <v>2016</v>
       </c>
       <c r="D66" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="F66" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="G66" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H66" s="1" t="s">
         <v>597</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>598</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>89</v>
       </c>
       <c r="J66" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="K66" s="1" t="s">
         <v>599</v>
       </c>
-      <c r="K66" s="1" t="s">
-        <v>600</v>
-      </c>
       <c r="X66" s="5" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="67" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="C67" s="1">
         <v>2015</v>
       </c>
       <c r="D67" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="E67" s="1" t="s">
         <v>601</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="F67" s="1" t="s">
         <v>602</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="G67" s="1" t="s">
         <v>603</v>
       </c>
-      <c r="G67" s="1" t="s">
+      <c r="H67" s="1" t="s">
         <v>604</v>
       </c>
-      <c r="H67" s="1" t="s">
+      <c r="J67" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="J67" s="1" t="s">
+      <c r="K67" s="1" t="s">
         <v>606</v>
       </c>
-      <c r="K67" s="1" t="s">
+      <c r="L67" s="1" t="s">
         <v>607</v>
       </c>
-      <c r="L67" s="1" t="s">
+      <c r="O67" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="O67" s="1" t="s">
+      <c r="X67" s="1" t="s">
         <v>609</v>
-      </c>
-      <c r="X67" s="1" t="s">
-        <v>610</v>
       </c>
     </row>
     <row r="68" spans="1:24" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C68" s="1">
         <v>2013</v>
       </c>
       <c r="D68" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>612</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="F68" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="F68" s="1" t="s">
+      <c r="G68" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="J68" s="1" t="s">
         <v>614</v>
       </c>
-      <c r="G68" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="J68" s="1" t="s">
+      <c r="K68" s="1" t="s">
         <v>615</v>
       </c>
-      <c r="K68" s="1" t="s">
-        <v>616</v>
-      </c>
       <c r="X68" s="5" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Starting add some articles in CN
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ghe/Documents/GitHub/drganghe.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{890B6DE5-0D0D-6A41-8CA0-420B20C46551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4EFAFD1-95CA-ED4C-9348-64997FBE0A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2376,7 +2376,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2406,6 +2406,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3581,11 +3585,17 @@
       <c r="E18" s="22" t="s">
         <v>684</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="28" t="s">
         <v>685</v>
       </c>
       <c r="G18" s="22" t="s">
         <v>686</v>
+      </c>
+      <c r="H18" s="27">
+        <v>7</v>
+      </c>
+      <c r="J18" s="27">
+        <v>533</v>
       </c>
       <c r="K18" s="22" t="s">
         <v>687</v>
@@ -5705,10 +5715,9 @@
     <hyperlink ref="R6" r:id="rId16" xr:uid="{3BA53A63-8360-5C4A-8B83-6B57EC2CA670}"/>
     <hyperlink ref="O24" r:id="rId17" xr:uid="{DBD76148-39E2-0A4A-BEB0-0119C38CF222}"/>
     <hyperlink ref="P19" r:id="rId18" xr:uid="{86409AA4-BEFD-D542-B873-480C74955AF8}"/>
-    <hyperlink ref="F18" r:id="rId19" xr:uid="{D215DD66-92F0-B743-B8A1-3D4196786705}"/>
-    <hyperlink ref="O18" r:id="rId20" xr:uid="{1D7B2550-014B-C64E-AEB9-00BD366191E0}"/>
-    <hyperlink ref="P18" r:id="rId21" xr:uid="{5DE482F3-CFB9-9F4D-9BDA-A163AE0ADB50}"/>
-    <hyperlink ref="R18" r:id="rId22" xr:uid="{BFAA4559-24D5-B443-8FC5-A54634E39487}"/>
+    <hyperlink ref="O18" r:id="rId19" xr:uid="{1D7B2550-014B-C64E-AEB9-00BD366191E0}"/>
+    <hyperlink ref="P18" r:id="rId20" xr:uid="{5DE482F3-CFB9-9F4D-9BDA-A163AE0ADB50}"/>
+    <hyperlink ref="R18" r:id="rId21" xr:uid="{BFAA4559-24D5-B443-8FC5-A54634E39487}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>